<commit_message>
updated WHO BAR estimate excel
</commit_message>
<xml_diff>
--- a/data_processing/assumptions_and_estimates/who_bar_reduction_to_cb_factors.xlsx
+++ b/data_processing/assumptions_and_estimates/who_bar_reduction_to_cb_factors.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/ssp_uganda_data/data_processing/assumptions_and_estimates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10245F6F-C300-2546-898C-7F616DAEF019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1D5DE0-7E2D-0D4A-AE13-F4680293B6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2820" yWindow="760" windowWidth="29020" windowHeight="16940" xr2:uid="{33EDD947-1184-1145-A09E-4DECC944BF75}"/>
+    <workbookView xWindow="4980" yWindow="760" windowWidth="29020" windowHeight="16940" xr2:uid="{33EDD947-1184-1145-A09E-4DECC944BF75}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="32">
   <si>
     <t>From J12 on Summary Setup</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>NOTE: IGNORE POLICIES WITH NEGATIVE NET BENEFIT PER CAPITA FOR OUR PURPOSES</t>
+  </si>
+  <si>
+    <t>hgl_to_electricity</t>
   </si>
 </sst>
 </file>
@@ -172,7 +175,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -209,6 +212,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -222,16 +231,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -243,6 +246,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -252,10 +265,12 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -590,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F022ABB-1E74-5E44-965B-6D32501E8D2C}">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
@@ -614,10 +629,10 @@
       <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -640,1077 +655,1527 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
         <f>B1*B2</f>
         <v>43826891.130000003</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="J5" s="6" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>27386330</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>6777500</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="3">
         <f>(D6-E6)/$B$3</f>
         <v>0.47023253232518297</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <f>F6*$J$2</f>
         <v>1.3494401179375923</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="2">
+      <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="8">
         <f>F7-F6</f>
         <v>1.191136917404253</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="8">
         <f>G7-G6</f>
         <v>3.4182406188567613</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>72812658</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3">
         <f t="shared" ref="F7:F45" si="0">(D7-E7)/$B$3</f>
         <v>1.661369449729436</v>
       </c>
-      <c r="G7" s="5">
-        <f t="shared" ref="G7:G45" si="1">F7*$J$2</f>
+      <c r="G7" s="3">
+        <f t="shared" ref="G7:G43" si="1">F7*$J$2</f>
         <v>4.7676807367943539</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="H7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>1582.8</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
         <v>3.611481351266906E-5</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="5" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>3592.3</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
         <v>8.1965658694440916E-5</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>50975422</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="5">
         <v>-1428886</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="5">
         <f>(D10-E10)/$B$3</f>
         <v>1.1957112779128578</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="5">
         <f t="shared" si="1"/>
         <v>3.4313677956467159</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="2">
+      <c r="H10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="8">
         <f>F11-F10</f>
         <v>0.66550018146358991</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="8">
         <f>G11-G10</f>
         <v>1.9098054294990372</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="7" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="5">
         <v>81571112</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7">
+      <c r="E11" s="5"/>
+      <c r="F11" s="5">
         <f>(D11-E11)/$B$3</f>
         <v>1.8612114593764477</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="5">
         <f t="shared" si="1"/>
         <v>5.3411732251457531</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
+      <c r="H11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="7" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="5">
         <v>1904.7</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7">
+      <c r="E12" s="5"/>
+      <c r="F12" s="5">
         <f t="shared" si="0"/>
         <v>4.3459619217576931E-5</v>
       </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="7" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="5">
         <v>4469</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7">
+      <c r="E13" s="5"/>
+      <c r="F13" s="5">
         <f t="shared" si="0"/>
         <v>1.0196935910293028E-4</v>
       </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="3">
         <v>69132794</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="3">
         <v>17690132</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="3">
         <f t="shared" si="0"/>
         <v>1.1737693610849553</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="3">
         <f t="shared" si="1"/>
         <v>3.3684004320625527</v>
       </c>
-      <c r="H14" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I14" s="2">
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="8">
         <f>F15-F14</f>
         <v>3.1626152215282626</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="8">
         <f>G15-G14</f>
         <v>9.0758498490678914</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="5" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="3">
         <v>190050255</v>
       </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3">
         <f t="shared" si="0"/>
         <v>4.3363845826132179</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="3">
         <f t="shared" si="1"/>
         <v>12.444250281130444</v>
       </c>
-      <c r="H15" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+      <c r="H15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="5" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="3">
         <v>4131.3999999999996</v>
       </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3">
         <f t="shared" si="0"/>
         <v>9.4266325844226027E-5</v>
       </c>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="5" t="s">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="3">
         <v>9376.4</v>
       </c>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3">
         <f t="shared" si="0"/>
         <v>2.1394170926218738E-4</v>
       </c>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="5">
         <v>1864991607</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="5">
         <v>70420222</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="5">
         <f t="shared" si="0"/>
         <v>40.946810023027062</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="5">
         <f t="shared" si="1"/>
         <v>117.50626413153141</v>
       </c>
-      <c r="H18" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I18" s="3">
+      <c r="H18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18" s="9">
         <f>F19-F18</f>
         <v>-23.798678713171135</v>
       </c>
-      <c r="J18" s="3">
+      <c r="J18" s="9">
         <f>G19-G18</f>
         <v>-68.29576773572083</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="7" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <v>751549284</v>
       </c>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7">
+      <c r="E19" s="5"/>
+      <c r="F19" s="5">
         <f t="shared" si="0"/>
         <v>17.148131309855927</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="5">
         <f t="shared" si="1"/>
         <v>49.210496395810587</v>
       </c>
-      <c r="H19" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="H19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="8"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="7" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="5">
         <v>7894.2</v>
       </c>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7">
+      <c r="E20" s="5"/>
+      <c r="F20" s="5">
         <f t="shared" si="0"/>
         <v>1.8012229013881229E-4</v>
       </c>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="8"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="7" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="5">
         <v>17916.099999999999</v>
       </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7">
+      <c r="E21" s="5"/>
+      <c r="F21" s="5">
         <f t="shared" si="0"/>
         <v>4.0879239978160864E-4</v>
       </c>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8" t="s">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="3">
         <v>40242617</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="3">
         <v>9505658</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="3">
         <f t="shared" si="0"/>
         <v>0.70132647348468224</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="3">
         <f t="shared" si="1"/>
         <v>2.0126171926306804</v>
       </c>
-      <c r="H22" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I22" s="2">
+      <c r="H22" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" s="8">
         <f>F23-F22</f>
         <v>1.6287967765784803</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="8">
         <f>G23-G22</f>
         <v>4.6742059793567474</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="5" t="s">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="3">
         <v>102122058</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5">
+      <c r="E23" s="3"/>
+      <c r="F23" s="3">
         <f t="shared" si="0"/>
         <v>2.3301232500631626</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="3">
         <f t="shared" si="1"/>
         <v>6.6868231719874274</v>
       </c>
-      <c r="H23" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+      <c r="H23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="5" t="s">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="3">
         <v>2220</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5">
+      <c r="E24" s="3"/>
+      <c r="F24" s="3">
         <f t="shared" si="0"/>
         <v>5.065383244764046E-5</v>
       </c>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="5" t="s">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="3">
         <v>5038.3</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5">
+      <c r="E25" s="3"/>
+      <c r="F25" s="3">
         <f t="shared" si="0"/>
         <v>1.1495910091033646E-4</v>
       </c>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="4">
         <v>-54741148</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="4">
         <v>-95360398</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="4">
         <f t="shared" si="0"/>
         <v>0.92681111876072964</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="4">
         <f t="shared" si="1"/>
         <v>2.6596971060723269</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I26" s="2">
+      <c r="H26" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="8">
         <f>F27-F26</f>
         <v>2.4066885028903942</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="8">
         <f>G27-G26</f>
         <v>6.9065447282443024</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="6" t="s">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="4">
         <v>146096925</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6">
+      <c r="E27" s="4"/>
+      <c r="F27" s="4">
         <f t="shared" si="0"/>
         <v>3.3334996216511237</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="4">
         <f t="shared" si="1"/>
         <v>9.5662418343166298</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+      <c r="H27" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="6" t="s">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="4">
         <v>3067.7</v>
       </c>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6">
+      <c r="E28" s="4"/>
+      <c r="F28" s="4">
         <f t="shared" si="0"/>
         <v>6.9995838648480465E-5</v>
       </c>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="6" t="s">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="4">
         <v>6980.4</v>
       </c>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6">
+      <c r="E29" s="4"/>
+      <c r="F29" s="4">
         <f t="shared" si="0"/>
         <v>1.592720774853646E-4</v>
       </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="10"/>
-      <c r="B30" s="9" t="s">
+      <c r="A30" s="12"/>
+      <c r="B30" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="5">
         <v>95137083</v>
       </c>
-      <c r="E30" s="7">
-        <v>0</v>
-      </c>
-      <c r="F30" s="7">
+      <c r="E30" s="5">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5">
         <f t="shared" si="0"/>
         <v>2.1707467846122808</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="5">
         <f t="shared" si="1"/>
         <v>6.2294558450799249</v>
       </c>
-      <c r="H30" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I30" s="2">
+      <c r="H30" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I30" s="8">
         <f>F31-F30</f>
         <v>1.7773993544040825</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="8">
         <f>G31-G30</f>
         <v>5.1006551643062403</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="10"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="7" t="s">
+      <c r="A31" s="12"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="5">
         <v>173034971</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7">
+      <c r="E31" s="5"/>
+      <c r="F31" s="5">
         <f t="shared" si="0"/>
         <v>3.9481461390163632</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="5">
         <f t="shared" si="1"/>
         <v>11.330111009386165</v>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+      <c r="H31" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="10"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="7" t="s">
+      <c r="A32" s="12"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="5">
         <v>3692.6</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7">
+      <c r="E32" s="5"/>
+      <c r="F32" s="5">
         <f t="shared" si="0"/>
         <v>8.4254207971241963E-5</v>
       </c>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="7" t="s">
+      <c r="A33" s="12"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="5">
         <v>8688.5</v>
       </c>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7">
+      <c r="E33" s="5"/>
+      <c r="F33" s="5">
         <f t="shared" si="0"/>
         <v>1.9824586631591177E-4</v>
       </c>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10" t="s">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="4">
         <v>-101164854</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="4">
         <v>-175057131</v>
       </c>
-      <c r="F34" s="6">
+      <c r="F34" s="4">
         <f t="shared" si="0"/>
         <v>1.6860031614110977</v>
       </c>
-      <c r="G34" s="6">
+      <c r="G34" s="4">
         <f t="shared" si="1"/>
         <v>4.8383728231809977</v>
       </c>
-      <c r="H34" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I34" s="2">
+      <c r="H34" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I34" s="8">
         <f>F35-F34</f>
         <v>4.4334435774523069</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="8">
         <f>G35-G34</f>
         <v>12.722783331140668</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="6" t="s">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="4">
         <v>268196326</v>
       </c>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6">
+      <c r="E35" s="4"/>
+      <c r="F35" s="4">
         <f t="shared" si="0"/>
         <v>6.1194467388634051</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="4">
         <f t="shared" si="1"/>
         <v>17.561156154321665</v>
       </c>
-      <c r="H35" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="H35" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="6" t="s">
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="4">
         <v>5631.5</v>
       </c>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6">
+      <c r="E36" s="4"/>
+      <c r="F36" s="4">
         <f t="shared" si="0"/>
         <v>1.2849417001301229E-4</v>
       </c>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="6" t="s">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="4">
         <v>12814.2</v>
       </c>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6">
+      <c r="E37" s="4"/>
+      <c r="F37" s="4">
         <f t="shared" si="0"/>
         <v>2.9238213502277225E-4</v>
       </c>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A38" s="10"/>
-      <c r="B38" s="9" t="s">
+      <c r="A38" s="12"/>
+      <c r="B38" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="5">
         <v>1216132864</v>
       </c>
-      <c r="E38" s="7">
+      <c r="E38" s="5">
         <v>-514290336</v>
       </c>
-      <c r="F38" s="7">
+      <c r="F38" s="5">
         <f t="shared" si="0"/>
         <v>39.483138214553982</v>
       </c>
-      <c r="G38" s="7">
+      <c r="G38" s="5">
         <f t="shared" si="1"/>
         <v>113.30592212609575</v>
       </c>
-      <c r="H38" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I38" s="3">
+      <c r="H38" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I38" s="9">
         <f>F39-F38</f>
         <v>-21.630713234666985</v>
       </c>
-      <c r="J38" s="3">
+      <c r="J38" s="9">
         <f>G39-G38</f>
         <v>-62.07429348652073</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A39" s="10"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="7" t="s">
+      <c r="A39" s="12"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="7">
+      <c r="D39" s="5">
         <v>782416286</v>
       </c>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7">
+      <c r="E39" s="5"/>
+      <c r="F39" s="5">
         <f t="shared" si="0"/>
         <v>17.852424979886997</v>
       </c>
-      <c r="G39" s="7">
+      <c r="G39" s="5">
         <f t="shared" si="1"/>
         <v>51.231628639575021</v>
       </c>
-      <c r="H39" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
+      <c r="H39" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A40" s="10"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="7" t="s">
+      <c r="A40" s="12"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D40" s="7">
+      <c r="D40" s="5">
         <v>7941.4</v>
       </c>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7">
+      <c r="E40" s="5"/>
+      <c r="F40" s="5">
         <f t="shared" si="0"/>
         <v>1.8119925450436574E-4</v>
       </c>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" s="10"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="7" t="s">
+      <c r="A41" s="12"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D41" s="7">
+      <c r="D41" s="5">
         <v>18070.099999999999</v>
       </c>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7">
+      <c r="E41" s="5"/>
+      <c r="F41" s="5">
         <f t="shared" si="0"/>
         <v>4.1230622419464314E-4</v>
       </c>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10" t="s">
+      <c r="A42" s="12"/>
+      <c r="B42" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D42" s="6">
+      <c r="D42" s="4">
         <v>-61287575</v>
       </c>
-      <c r="E42" s="6">
+      <c r="E42" s="4">
         <v>-115284582</v>
       </c>
-      <c r="F42" s="6">
+      <c r="F42" s="4">
         <f t="shared" si="0"/>
         <v>1.2320519573207518</v>
       </c>
-      <c r="G42" s="6">
+      <c r="G42" s="4">
         <f t="shared" si="1"/>
         <v>3.5356557113798792</v>
       </c>
-      <c r="H42" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I42" s="2">
+      <c r="H42" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I42" s="8">
         <f>F43-F42</f>
         <v>2.7979344379291815</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="8">
         <f>G43-G42</f>
         <v>8.0293146865683251</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="6" t="s">
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="4">
         <v>176621775</v>
       </c>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6">
+      <c r="E43" s="4"/>
+      <c r="F43" s="4">
         <f t="shared" si="0"/>
         <v>4.0299863952499333</v>
       </c>
-      <c r="G43" s="6">
+      <c r="G43" s="4">
         <f t="shared" si="1"/>
         <v>11.564970397948205</v>
       </c>
-      <c r="H43" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I43" s="2"/>
-      <c r="J43" s="2"/>
+      <c r="H43" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" s="10"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="6" t="s">
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D44" s="6">
+      <c r="D44" s="4">
         <v>3708.7</v>
       </c>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6">
+      <c r="E44" s="4"/>
+      <c r="F44" s="4">
         <f t="shared" si="0"/>
         <v>8.4621562341695563E-5</v>
       </c>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I44" s="8"/>
+      <c r="J44" s="8"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="6" t="s">
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D45" s="6">
+      <c r="D45" s="4">
         <v>8438.7999999999993</v>
       </c>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6">
+      <c r="E45" s="4"/>
+      <c r="F45" s="4">
         <f t="shared" si="0"/>
         <v>1.9254845101763436E-4</v>
       </c>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I45" s="8"/>
+      <c r="J45" s="8"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14">
+        <f t="shared" ref="F46:F65" si="2">(D46-E46)/$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="14">
+        <f t="shared" ref="G46:G47" si="3">F46*$J$2</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I46" s="8">
+        <f>F47-F46</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="8">
+        <f>G47-G46</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" s="13"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G47" s="14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H47" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I47" s="8"/>
+      <c r="J47" s="8"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" s="13"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G48" s="14"/>
+      <c r="H48" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I48" s="8"/>
+      <c r="J48" s="8"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" s="13"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G49" s="14"/>
+      <c r="H49" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" s="13"/>
+      <c r="B50" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5">
+        <v>0</v>
+      </c>
+      <c r="F50" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="5">
+        <f t="shared" ref="G50:G51" si="4">F50*$J$2</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I50" s="8">
+        <f>F51-F50</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="8">
+        <f>G51-G50</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" s="13"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G51" s="5">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I51" s="8"/>
+      <c r="J51" s="8"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" s="13"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I52" s="8"/>
+      <c r="J52" s="8"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A53" s="13"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I53" s="8"/>
+      <c r="J53" s="8"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A54" s="13"/>
+      <c r="B54" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="14">
+        <f t="shared" ref="G54:G55" si="5">F54*$J$2</f>
+        <v>0</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I54" s="8">
+        <f>F55-F54</f>
+        <v>0</v>
+      </c>
+      <c r="J54" s="8">
+        <f>G55-G54</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A55" s="13"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G55" s="14">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H55" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I55" s="8"/>
+      <c r="J55" s="8"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A56" s="13"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G56" s="14"/>
+      <c r="H56" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I56" s="8"/>
+      <c r="J56" s="8"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A57" s="13"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G57" s="14"/>
+      <c r="H57" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A58" s="13"/>
+      <c r="B58" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G58" s="5">
+        <f t="shared" ref="G58:G59" si="6">F58*$J$2</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I58" s="9">
+        <f>F59-F58</f>
+        <v>0</v>
+      </c>
+      <c r="J58" s="9">
+        <f>G59-G58</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A59" s="13"/>
+      <c r="B59" s="11"/>
+      <c r="C59" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G59" s="5">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I59" s="9"/>
+      <c r="J59" s="9"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A60" s="13"/>
+      <c r="B60" s="11"/>
+      <c r="C60" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I60" s="9"/>
+      <c r="J60" s="9"/>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A61" s="13"/>
+      <c r="B61" s="11"/>
+      <c r="C61" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I61" s="9"/>
+      <c r="J61" s="9"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A62" s="13"/>
+      <c r="B62" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G62" s="14">
+        <f t="shared" ref="G62:G63" si="7">F62*$J$2</f>
+        <v>0</v>
+      </c>
+      <c r="H62" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I62" s="8">
+        <f>F63-F62</f>
+        <v>0</v>
+      </c>
+      <c r="J62" s="8">
+        <f>G63-G62</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A63" s="13"/>
+      <c r="B63" s="13"/>
+      <c r="C63" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G63" s="14">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="H63" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I63" s="8"/>
+      <c r="J63" s="8"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A64" s="13"/>
+      <c r="B64" s="13"/>
+      <c r="C64" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G64" s="14"/>
+      <c r="H64" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I64" s="8"/>
+      <c r="J64" s="8"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A65" s="13"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G65" s="14"/>
+      <c r="H65" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I65" s="8"/>
+      <c r="J65" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="J30:J33"/>
-    <mergeCell ref="J34:J37"/>
-    <mergeCell ref="J38:J41"/>
-    <mergeCell ref="J42:J45"/>
-    <mergeCell ref="I30:I33"/>
-    <mergeCell ref="I34:I37"/>
-    <mergeCell ref="I38:I41"/>
-    <mergeCell ref="I42:I45"/>
-    <mergeCell ref="J6:J9"/>
-    <mergeCell ref="J10:J13"/>
-    <mergeCell ref="J14:J17"/>
-    <mergeCell ref="J18:J21"/>
-    <mergeCell ref="J22:J25"/>
-    <mergeCell ref="J26:J29"/>
-    <mergeCell ref="I6:I9"/>
-    <mergeCell ref="I10:I13"/>
-    <mergeCell ref="I14:I17"/>
-    <mergeCell ref="I18:I21"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I26:I29"/>
+  <mergeCells count="48">
+    <mergeCell ref="A46:A65"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="I46:I49"/>
+    <mergeCell ref="J46:J49"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="I50:I53"/>
+    <mergeCell ref="J50:J53"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="I54:I57"/>
+    <mergeCell ref="J54:J57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="I58:I61"/>
+    <mergeCell ref="J58:J61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="I62:I65"/>
+    <mergeCell ref="J62:J65"/>
     <mergeCell ref="B14:B17"/>
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="B22:B25"/>
@@ -1723,6 +2188,26 @@
     <mergeCell ref="B42:B45"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="B10:B13"/>
+    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="I6:I9"/>
+    <mergeCell ref="I10:I13"/>
+    <mergeCell ref="I14:I17"/>
+    <mergeCell ref="I18:I21"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="I26:I29"/>
+    <mergeCell ref="J6:J9"/>
+    <mergeCell ref="J10:J13"/>
+    <mergeCell ref="J14:J17"/>
+    <mergeCell ref="J18:J21"/>
+    <mergeCell ref="J22:J25"/>
+    <mergeCell ref="J30:J33"/>
+    <mergeCell ref="J34:J37"/>
+    <mergeCell ref="J38:J41"/>
+    <mergeCell ref="J42:J45"/>
+    <mergeCell ref="I30:I33"/>
+    <mergeCell ref="I34:I37"/>
+    <mergeCell ref="I38:I41"/>
+    <mergeCell ref="I42:I45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>